<commit_message>
BestBuy - logs updated, asserts added
</commit_message>
<xml_diff>
--- a/SeleniumPytest/BestBuy/test_data/test_data.xlsx
+++ b/SeleniumPytest/BestBuy/test_data/test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayush\OneDrive\Desktop\WiproCapstoneProject\SeleniumPytest\BestBuy\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EEED1F-DBAA-4493-9FBC-11E4939AE49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{072F3C8A-2260-4CCF-BB3C-D68B9409B61F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BrandFilters" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Samsung</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t>abc#xyz.com</t>
+  </si>
+  <si>
+    <t>brand</t>
   </si>
 </sst>
 </file>
@@ -398,34 +401,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -460,7 +465,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD2D8C3F-EB5B-480E-9C41-599F18780837}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" customWidth="1"/>
@@ -480,6 +485,14 @@
       </c>
       <c r="B2">
         <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3276378</v>
+      </c>
+      <c r="B3">
+        <v>2397892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>